<commit_message>
fix(resumen): mapear items piques nuevos + forzar fullCalcOnLoad
Dos bugs detectados al revisar Resumen Oferta:

1. Items 4.x.4 a 4.x.7 y 4.x.9 (suma alzada piques) tenian precio
   en col E pero D (cantidad) quedaba None. Causa: _PIQUE_ITEMS
   mapping no incluia las claves nuevas. Resultado: cant=None ×
   precio = 0 en col F. Fix: agregar las 5 claves al mapeo.

2. Resumen Oferta mostraba celdas vacias al abrir el xlsx generado
   por openpyxl porque las formulas no tienen valor cacheado. Fix:
   activar wb.calculation.fullCalcOnLoad = True para que Excel
   recalcule todas las formulas al abrir.

Verificacion manual:
- Pique 1 subtotal: 1,519 UF (todos los items con cant llenada)
- A) Total Costo Directo: 77,601 UF (antes era 74,843)
- B) Total Indirecto: 31,680 UF
- B) Total GG: 6,200 UF
- B) Total Utilidad: 8,000 UF
- Total Neto: 123,481 UF
- IVA: 23,461 UF
- TOTAL: 146,943 UF (~$5,657M CLP)

https://claude.ai/code/session_016BR4zVrkucAbqsHCWRUVRh
</commit_message>
<xml_diff>
--- a/output/licitacion_vitacura.xlsx
+++ b/output/licitacion_vitacura.xlsx
@@ -3155,12 +3155,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D45" s="49" t="n"/>
+      <c r="D45" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E45" s="222" t="n">
         <v>72.7273</v>
       </c>
-      <c r="F45" s="210">
-        <f>+D45*E45</f>
+      <c r="F45" s="205">
+        <f>D45*E45</f>
         <v/>
       </c>
       <c r="G45" s="47" t="inlineStr">
@@ -3186,12 +3188,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D46" s="49" t="n"/>
+      <c r="D46" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E46" s="222" t="n">
         <v>46.7532</v>
       </c>
-      <c r="F46" s="210">
-        <f>+D46*E46</f>
+      <c r="F46" s="205">
+        <f>D46*E46</f>
         <v/>
       </c>
       <c r="G46" s="47" t="inlineStr">
@@ -3217,12 +3221,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D47" s="49" t="n"/>
+      <c r="D47" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E47" s="222" t="n">
         <v>38.961</v>
       </c>
-      <c r="F47" s="210">
-        <f>+D47*E47</f>
+      <c r="F47" s="205">
+        <f>D47*E47</f>
         <v/>
       </c>
       <c r="G47" s="47" t="inlineStr">
@@ -3248,12 +3254,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D48" s="49" t="n"/>
+      <c r="D48" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E48" s="222" t="n">
         <v>90.9091</v>
       </c>
-      <c r="F48" s="210">
-        <f>+D48*E48</f>
+      <c r="F48" s="205">
+        <f>D48*E48</f>
         <v/>
       </c>
       <c r="G48" s="47" t="inlineStr">
@@ -3312,12 +3320,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D50" s="49" t="n"/>
+      <c r="D50" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E50" s="222" t="n">
         <v>57.1429</v>
       </c>
-      <c r="F50" s="210">
-        <f>+D50*E50</f>
+      <c r="F50" s="205">
+        <f>D50*E50</f>
         <v/>
       </c>
       <c r="G50" s="47" t="inlineStr">
@@ -3667,12 +3677,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D62" s="49" t="n"/>
+      <c r="D62" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E62" s="222" t="n">
         <v>72.7273</v>
       </c>
-      <c r="F62" s="210">
-        <f>+D62*E62</f>
+      <c r="F62" s="205">
+        <f>D62*E62</f>
         <v/>
       </c>
       <c r="G62" s="47" t="inlineStr">
@@ -3698,12 +3710,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D63" s="49" t="n"/>
+      <c r="D63" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E63" s="222" t="n">
         <v>46.7532</v>
       </c>
-      <c r="F63" s="210">
-        <f>+D63*E63</f>
+      <c r="F63" s="205">
+        <f>D63*E63</f>
         <v/>
       </c>
       <c r="G63" s="47" t="inlineStr">
@@ -3729,12 +3743,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D64" s="49" t="n"/>
+      <c r="D64" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E64" s="222" t="n">
         <v>38.961</v>
       </c>
-      <c r="F64" s="210">
-        <f>+D64*E64</f>
+      <c r="F64" s="205">
+        <f>D64*E64</f>
         <v/>
       </c>
       <c r="G64" s="47" t="inlineStr">
@@ -3760,12 +3776,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D65" s="49" t="n"/>
+      <c r="D65" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E65" s="222" t="n">
         <v>90.9091</v>
       </c>
-      <c r="F65" s="210">
-        <f>+D65*E65</f>
+      <c r="F65" s="205">
+        <f>D65*E65</f>
         <v/>
       </c>
       <c r="G65" s="47" t="inlineStr">
@@ -3824,12 +3842,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D67" s="49" t="n"/>
+      <c r="D67" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E67" s="222" t="n">
         <v>57.1429</v>
       </c>
-      <c r="F67" s="210">
-        <f>+D67*E67</f>
+      <c r="F67" s="205">
+        <f>D67*E67</f>
         <v/>
       </c>
       <c r="G67" s="47" t="inlineStr">
@@ -4146,12 +4166,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D78" s="49" t="n"/>
+      <c r="D78" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E78" s="222" t="n">
         <v>72.7273</v>
       </c>
-      <c r="F78" s="210">
-        <f>+D78*E78</f>
+      <c r="F78" s="205">
+        <f>D78*E78</f>
         <v/>
       </c>
       <c r="G78" s="47" t="inlineStr">
@@ -4177,12 +4199,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D79" s="49" t="n"/>
+      <c r="D79" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E79" s="222" t="n">
         <v>46.7532</v>
       </c>
-      <c r="F79" s="210">
-        <f>+D79*E79</f>
+      <c r="F79" s="205">
+        <f>D79*E79</f>
         <v/>
       </c>
       <c r="G79" s="47" t="inlineStr">
@@ -4208,12 +4232,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D80" s="49" t="n"/>
+      <c r="D80" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E80" s="222" t="n">
         <v>38.961</v>
       </c>
-      <c r="F80" s="210">
-        <f>+D80*E80</f>
+      <c r="F80" s="205">
+        <f>D80*E80</f>
         <v/>
       </c>
       <c r="G80" s="47" t="inlineStr">
@@ -4239,12 +4265,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D81" s="49" t="n"/>
+      <c r="D81" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E81" s="222" t="n">
         <v>90.9091</v>
       </c>
-      <c r="F81" s="210">
-        <f>+D81*E81</f>
+      <c r="F81" s="205">
+        <f>D81*E81</f>
         <v/>
       </c>
       <c r="G81" s="47" t="inlineStr">
@@ -4303,12 +4331,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D83" s="49" t="n"/>
+      <c r="D83" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E83" s="222" t="n">
         <v>57.1429</v>
       </c>
-      <c r="F83" s="210">
-        <f>+D83*E83</f>
+      <c r="F83" s="205">
+        <f>D83*E83</f>
         <v/>
       </c>
       <c r="G83" s="47" t="inlineStr">
@@ -4625,12 +4655,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D94" s="49" t="n"/>
+      <c r="D94" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E94" s="222" t="n">
         <v>72.7273</v>
       </c>
-      <c r="F94" s="210">
-        <f>+D94*E94</f>
+      <c r="F94" s="205">
+        <f>D94*E94</f>
         <v/>
       </c>
       <c r="G94" s="47" t="inlineStr">
@@ -4656,12 +4688,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D95" s="49" t="n"/>
+      <c r="D95" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E95" s="222" t="n">
         <v>46.7532</v>
       </c>
-      <c r="F95" s="210">
-        <f>+D95*E95</f>
+      <c r="F95" s="205">
+        <f>D95*E95</f>
         <v/>
       </c>
       <c r="G95" s="47" t="inlineStr">
@@ -4687,12 +4721,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D96" s="49" t="n"/>
+      <c r="D96" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E96" s="222" t="n">
         <v>38.961</v>
       </c>
-      <c r="F96" s="210">
-        <f>+D96*E96</f>
+      <c r="F96" s="205">
+        <f>D96*E96</f>
         <v/>
       </c>
       <c r="G96" s="47" t="inlineStr">
@@ -4718,12 +4754,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D97" s="49" t="n"/>
+      <c r="D97" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E97" s="222" t="n">
         <v>90.9091</v>
       </c>
-      <c r="F97" s="210">
-        <f>+D97*E97</f>
+      <c r="F97" s="205">
+        <f>D97*E97</f>
         <v/>
       </c>
       <c r="G97" s="47" t="inlineStr">
@@ -4782,12 +4820,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D99" s="49" t="n"/>
+      <c r="D99" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E99" s="222" t="n">
         <v>57.1429</v>
       </c>
-      <c r="F99" s="210">
-        <f>+D99*E99</f>
+      <c r="F99" s="205">
+        <f>D99*E99</f>
         <v/>
       </c>
       <c r="G99" s="47" t="inlineStr">
@@ -5104,12 +5144,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D110" s="49" t="n"/>
+      <c r="D110" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E110" s="222" t="n">
         <v>72.7273</v>
       </c>
-      <c r="F110" s="210">
-        <f>+D110*E110</f>
+      <c r="F110" s="205">
+        <f>D110*E110</f>
         <v/>
       </c>
       <c r="G110" s="47" t="inlineStr">
@@ -5135,12 +5177,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D111" s="49" t="n"/>
+      <c r="D111" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E111" s="222" t="n">
         <v>46.7532</v>
       </c>
-      <c r="F111" s="210">
-        <f>+D111*E111</f>
+      <c r="F111" s="205">
+        <f>D111*E111</f>
         <v/>
       </c>
       <c r="G111" s="47" t="inlineStr">
@@ -5166,12 +5210,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D112" s="49" t="n"/>
+      <c r="D112" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E112" s="222" t="n">
         <v>38.961</v>
       </c>
-      <c r="F112" s="210">
-        <f>+D112*E112</f>
+      <c r="F112" s="205">
+        <f>D112*E112</f>
         <v/>
       </c>
       <c r="G112" s="47" t="inlineStr">
@@ -5197,12 +5243,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D113" s="49" t="n"/>
+      <c r="D113" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E113" s="222" t="n">
         <v>90.9091</v>
       </c>
-      <c r="F113" s="210">
-        <f>+D113*E113</f>
+      <c r="F113" s="205">
+        <f>D113*E113</f>
         <v/>
       </c>
       <c r="G113" s="47" t="inlineStr">
@@ -5261,12 +5309,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D115" s="49" t="n"/>
+      <c r="D115" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E115" s="222" t="n">
         <v>57.1429</v>
       </c>
-      <c r="F115" s="210">
-        <f>+D115*E115</f>
+      <c r="F115" s="205">
+        <f>D115*E115</f>
         <v/>
       </c>
       <c r="G115" s="47" t="inlineStr">
@@ -5583,12 +5633,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D126" s="49" t="n"/>
+      <c r="D126" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E126" s="222" t="n">
         <v>72.7273</v>
       </c>
-      <c r="F126" s="210">
-        <f>+D126*E126</f>
+      <c r="F126" s="205">
+        <f>D126*E126</f>
         <v/>
       </c>
       <c r="G126" s="47" t="inlineStr">
@@ -5614,12 +5666,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D127" s="49" t="n"/>
+      <c r="D127" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E127" s="222" t="n">
         <v>46.7532</v>
       </c>
-      <c r="F127" s="210">
-        <f>+D127*E127</f>
+      <c r="F127" s="205">
+        <f>D127*E127</f>
         <v/>
       </c>
       <c r="G127" s="47" t="inlineStr">
@@ -5645,12 +5699,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D128" s="49" t="n"/>
+      <c r="D128" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E128" s="222" t="n">
         <v>38.961</v>
       </c>
-      <c r="F128" s="210">
-        <f>+D128*E128</f>
+      <c r="F128" s="205">
+        <f>D128*E128</f>
         <v/>
       </c>
       <c r="G128" s="47" t="inlineStr">
@@ -5676,12 +5732,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D129" s="49" t="n"/>
+      <c r="D129" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E129" s="222" t="n">
         <v>90.9091</v>
       </c>
-      <c r="F129" s="210">
-        <f>+D129*E129</f>
+      <c r="F129" s="205">
+        <f>D129*E129</f>
         <v/>
       </c>
       <c r="G129" s="47" t="inlineStr">
@@ -5740,12 +5798,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D131" s="49" t="n"/>
+      <c r="D131" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E131" s="222" t="n">
         <v>57.1429</v>
       </c>
-      <c r="F131" s="210">
-        <f>+D131*E131</f>
+      <c r="F131" s="205">
+        <f>D131*E131</f>
         <v/>
       </c>
       <c r="G131" s="47" t="inlineStr">
@@ -6062,12 +6122,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D142" s="49" t="n"/>
+      <c r="D142" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E142" s="222" t="n">
         <v>72.7273</v>
       </c>
-      <c r="F142" s="210">
-        <f>+D142*E142</f>
+      <c r="F142" s="205">
+        <f>D142*E142</f>
         <v/>
       </c>
       <c r="G142" s="47" t="inlineStr">
@@ -6093,12 +6155,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D143" s="49" t="n"/>
+      <c r="D143" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E143" s="222" t="n">
         <v>46.7532</v>
       </c>
-      <c r="F143" s="210">
-        <f>+D143*E143</f>
+      <c r="F143" s="205">
+        <f>D143*E143</f>
         <v/>
       </c>
       <c r="G143" s="47" t="inlineStr">
@@ -6124,12 +6188,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D144" s="49" t="n"/>
+      <c r="D144" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E144" s="222" t="n">
         <v>38.961</v>
       </c>
-      <c r="F144" s="210">
-        <f>+D144*E144</f>
+      <c r="F144" s="205">
+        <f>D144*E144</f>
         <v/>
       </c>
       <c r="G144" s="47" t="inlineStr">
@@ -6155,12 +6221,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D145" s="49" t="n"/>
+      <c r="D145" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E145" s="222" t="n">
         <v>90.9091</v>
       </c>
-      <c r="F145" s="210">
-        <f>+D145*E145</f>
+      <c r="F145" s="205">
+        <f>D145*E145</f>
         <v/>
       </c>
       <c r="G145" s="47" t="inlineStr">
@@ -6219,12 +6287,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D147" s="49" t="n"/>
+      <c r="D147" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E147" s="222" t="n">
         <v>57.1429</v>
       </c>
-      <c r="F147" s="210">
-        <f>+D147*E147</f>
+      <c r="F147" s="205">
+        <f>D147*E147</f>
         <v/>
       </c>
       <c r="G147" s="47" t="inlineStr">
@@ -6541,12 +6611,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D158" s="49" t="n"/>
+      <c r="D158" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E158" s="222" t="n">
         <v>72.7273</v>
       </c>
-      <c r="F158" s="210">
-        <f>+D158*E158</f>
+      <c r="F158" s="205">
+        <f>D158*E158</f>
         <v/>
       </c>
       <c r="G158" s="47" t="inlineStr">
@@ -6572,12 +6644,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D159" s="49" t="n"/>
+      <c r="D159" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E159" s="222" t="n">
         <v>46.7532</v>
       </c>
-      <c r="F159" s="210">
-        <f>+D159*E159</f>
+      <c r="F159" s="205">
+        <f>D159*E159</f>
         <v/>
       </c>
       <c r="G159" s="47" t="inlineStr">
@@ -6603,12 +6677,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D160" s="49" t="n"/>
+      <c r="D160" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E160" s="222" t="n">
         <v>38.961</v>
       </c>
-      <c r="F160" s="210">
-        <f>+D160*E160</f>
+      <c r="F160" s="205">
+        <f>D160*E160</f>
         <v/>
       </c>
       <c r="G160" s="47" t="inlineStr">
@@ -6634,12 +6710,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D161" s="49" t="n"/>
+      <c r="D161" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E161" s="222" t="n">
         <v>90.9091</v>
       </c>
-      <c r="F161" s="210">
-        <f>+D161*E161</f>
+      <c r="F161" s="205">
+        <f>D161*E161</f>
         <v/>
       </c>
       <c r="G161" s="47" t="inlineStr">
@@ -6698,12 +6776,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D163" s="49" t="n"/>
+      <c r="D163" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E163" s="222" t="n">
         <v>57.1429</v>
       </c>
-      <c r="F163" s="210">
-        <f>+D163*E163</f>
+      <c r="F163" s="205">
+        <f>D163*E163</f>
         <v/>
       </c>
       <c r="G163" s="47" t="inlineStr">
@@ -7020,12 +7100,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D174" s="49" t="n"/>
+      <c r="D174" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E174" s="222" t="n">
         <v>72.7273</v>
       </c>
-      <c r="F174" s="210">
-        <f>+D174*E174</f>
+      <c r="F174" s="205">
+        <f>D174*E174</f>
         <v/>
       </c>
       <c r="G174" s="47" t="inlineStr">
@@ -7051,12 +7133,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D175" s="49" t="n"/>
+      <c r="D175" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E175" s="222" t="n">
         <v>46.7532</v>
       </c>
-      <c r="F175" s="210">
-        <f>+D175*E175</f>
+      <c r="F175" s="205">
+        <f>D175*E175</f>
         <v/>
       </c>
       <c r="G175" s="47" t="inlineStr">
@@ -7082,12 +7166,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D176" s="49" t="n"/>
+      <c r="D176" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E176" s="222" t="n">
         <v>38.961</v>
       </c>
-      <c r="F176" s="210">
-        <f>+D176*E176</f>
+      <c r="F176" s="205">
+        <f>D176*E176</f>
         <v/>
       </c>
       <c r="G176" s="47" t="inlineStr">
@@ -7113,12 +7199,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D177" s="49" t="n"/>
+      <c r="D177" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E177" s="222" t="n">
         <v>90.9091</v>
       </c>
-      <c r="F177" s="210">
-        <f>+D177*E177</f>
+      <c r="F177" s="205">
+        <f>D177*E177</f>
         <v/>
       </c>
       <c r="G177" s="47" t="inlineStr">
@@ -7177,12 +7265,14 @@
           <t>gl</t>
         </is>
       </c>
-      <c r="D179" s="49" t="n"/>
+      <c r="D179" s="221" t="n">
+        <v>1</v>
+      </c>
       <c r="E179" s="222" t="n">
         <v>57.1429</v>
       </c>
-      <c r="F179" s="210">
-        <f>+D179*E179</f>
+      <c r="F179" s="205">
+        <f>D179*E179</f>
         <v/>
       </c>
       <c r="G179" s="47" t="inlineStr">

</xml_diff>